<commit_message>
added or modified data
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2494600_cognizant_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\diet-fitness-planner-testing\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{1C02D53C-3943-437D-AD06-9C72BFEB35A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA233136-D02E-46BC-8459-8A750927891C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29922639-9C50-4C52-BE03-2E299BDF4907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E79C43E6-4882-47E7-AD56-902C06E4923F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">Username </t>
   </si>
@@ -50,10 +50,13 @@
     <t>user1</t>
   </si>
   <si>
-    <t>Pass123</t>
-  </si>
-  <si>
-    <t>user2</t>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>pass123</t>
   </si>
 </sst>
 </file>
@@ -438,18 +441,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>